<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-01
</commit_message>
<xml_diff>
--- a/A_Swing_Pattern.xlsx
+++ b/A_Swing_Pattern.xlsx
@@ -6091,7 +6091,7 @@
         <v>5.849</v>
       </c>
       <c r="AL47" s="2" t="n">
-        <v>5.838</v>
+        <v>5.839</v>
       </c>
       <c r="AM47" s="2" t="n">
         <v>5.591</v>
@@ -7298,7 +7298,7 @@
       <c r="L58" s="2" t="inlineStr"/>
       <c r="M58" s="2" t="inlineStr"/>
       <c r="N58" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O58" s="2" t="inlineStr"/>
       <c r="P58" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (HK/A/ETF) 2026-10-07
</commit_message>
<xml_diff>
--- a/A_Swing_Pattern.xlsx
+++ b/A_Swing_Pattern.xlsx
@@ -6321,7 +6321,7 @@
         <v>5.849</v>
       </c>
       <c r="AL49" s="2" t="n">
-        <v>5.838</v>
+        <v>5.839</v>
       </c>
       <c r="AM49" s="2" t="n">
         <v>5.591</v>
@@ -58455,7 +58455,7 @@
         <v>271.261</v>
       </c>
       <c r="AO494" s="2" t="n">
-        <v>257.116</v>
+        <v>257.115</v>
       </c>
       <c r="AP494" s="2" t="n">
         <v>259.71</v>

</xml_diff>